<commit_message>
import pump do not remove NaN
</commit_message>
<xml_diff>
--- a/inputExpConfig.xlsx
+++ b/inputExpConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AD084B3-85CA-4F5C-99AF-0654A55DEED9}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEE287D7-25DA-4AED-9420-AA00B0DF72D0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,10 +57,10 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_He-Xe-T20.xlsx</t>
-  </si>
-  <si>
-    <t>results/exp_He-Xe-T20-V/</t>
+    <t>input/input_exp_He-Xe-vs-H2-CG.xlsx</t>
+  </si>
+  <si>
+    <t>results/exp_He-Xe-vs-H2-CG</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes of main code before submitting paper
</commit_message>
<xml_diff>
--- a/inputExpConfig.xlsx
+++ b/inputExpConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEE287D7-25DA-4AED-9420-AA00B0DF72D0}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB44E106-96D9-4DF7-98A6-BDBE80A5AB40}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,10 +57,10 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_He-Xe-vs-H2-CG.xlsx</t>
-  </si>
-  <si>
-    <t>results/exp_He-Xe-vs-H2-CG</t>
+    <t>input/input_exp_H2-CO2-T32-P1500.xlsx</t>
+  </si>
+  <si>
+    <t>results/exp_H2-CO2-T32-P1500-H/</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update inputExpConfig.xlsx: modify configuration file to reflect recent changes in data structure.
</commit_message>
<xml_diff>
--- a/inputExpConfig.xlsx
+++ b/inputExpConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A66FE56-F6A8-4136-9913-49C1E63099B1}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{904B1D24-40C0-4166-990D-D9BFEBE0C55F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,10 +68,10 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_H2-CG-T40-P1160.xlsx</t>
-  </si>
-  <si>
-    <t>results/exp_H2-CG-T40-P1160-V/</t>
+    <t>input/input_exp_He-Xe-vs-H2-CGs.xlsx</t>
+  </si>
+  <si>
+    <t>results/exp_He-Xe-vs-H2-CGs/</t>
   </si>
 </sst>
 </file>
@@ -390,17 +390,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="32.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" customWidth="1"/>
-    <col min="6" max="6" width="32.85546875" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" customWidth="1"/>
+    <col min="3" max="3" width="32.88671875" customWidth="1"/>
+    <col min="4" max="4" width="25.109375" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="6" max="6" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -420,7 +420,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update inputExpConfig.xlsx: modify configuration to align with recent data structure changes.
</commit_message>
<xml_diff>
--- a/inputExpConfig.xlsx
+++ b/inputExpConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{904B1D24-40C0-4166-990D-D9BFEBE0C55F}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F98A41F1-2509-47D0-BFAD-C10F17AFC087}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="21600" windowHeight="11292" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,10 +68,10 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_He-Xe-vs-H2-CGs.xlsx</t>
-  </si>
-  <si>
-    <t>results/exp_He-Xe-vs-H2-CGs/</t>
+    <t>input/input_exp_He-CO2-T40-P1500-H.xlsx</t>
+  </si>
+  <si>
+    <t>results/exp_He-CO2-T40-P1500-H_AfterComps/</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update inputExpConfig.xlsx to reflect changes in experimental configuration settings
</commit_message>
<xml_diff>
--- a/inputExpConfig.xlsx
+++ b/inputExpConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{904B1D24-40C0-4166-990D-D9BFEBE0C55F}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC76B6E5-B426-4AFF-947B-730146F79F31}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="405" yWindow="2145" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,10 +68,10 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_He-Xe-vs-H2-CGs.xlsx</t>
-  </si>
-  <si>
-    <t>results/exp_He-Xe-vs-H2-CGs/</t>
+    <t>results/exp_H2-CO2-T32-P1500-Q2-H/</t>
+  </si>
+  <si>
+    <t>input/input_exp_H2-CO2-T32-P1500-Q2-H.xlsx</t>
   </si>
 </sst>
 </file>
@@ -390,17 +390,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26.88671875" customWidth="1"/>
-    <col min="3" max="3" width="32.88671875" customWidth="1"/>
-    <col min="4" max="4" width="25.109375" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
-    <col min="6" max="6" width="32.88671875" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="32.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" customWidth="1"/>
+    <col min="6" max="6" width="32.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -420,15 +420,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>

</xml_diff>